<commit_message>
At home work prepping and processing Nektar Data and fitting veinous data
</commit_message>
<xml_diff>
--- a/NektarMap.xlsx
+++ b/NektarMap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbnor\Documents\Full Body Flow Model Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2F95E9C-9EBA-4D1B-9657-A5AE1E0DCF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5964067-B7C6-4705-9808-043AEBEC9A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9CFF2691-E43C-4CC8-A4D8-65AD8583F44E}"/>
+    <workbookView xWindow="-21697" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{9CFF2691-E43C-4CC8-A4D8-65AD8583F44E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -134,9 +134,6 @@
     <t>length (cm)</t>
   </si>
   <si>
-    <t>2,3,4,5,6,1,2</t>
-  </si>
-  <si>
     <t>arteries27</t>
   </si>
   <si>
@@ -153,6 +150,9 @@
   </si>
   <si>
     <t>crop</t>
+  </si>
+  <si>
+    <t>Crop</t>
   </si>
 </sst>
 </file>
@@ -561,6 +561,9 @@
       <c r="E1" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -615,7 +618,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B5">
         <f>3.9+48.5</f>
@@ -671,9 +674,7 @@
       <c r="C8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>32</v>
-      </c>
+      <c r="D8" s="4"/>
       <c r="E8" s="4">
         <f>0.26+0.06+0.57+7.91+3.57+6.89+11.75</f>
         <v>31.01</v>
@@ -747,7 +748,7 @@
         <v>40.159999999999997</v>
       </c>
       <c r="F12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -795,7 +796,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B16">
         <f>16+20.5</f>
@@ -821,9 +822,7 @@
       <c r="C17" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="4">
-        <v>0</v>
-      </c>
+      <c r="D17" s="4"/>
       <c r="E17" s="4">
         <v>21.87</v>
       </c>
@@ -843,7 +842,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <f>6+12</f>
@@ -978,7 +977,7 @@
         <v>39.4</v>
       </c>
       <c r="F26" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1004,9 +1003,7 @@
       <c r="C28" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D28" s="3">
-        <v>4</v>
-      </c>
+      <c r="D28" s="3"/>
       <c r="E28" s="3">
         <v>1.27</v>
       </c>
@@ -1130,7 +1127,7 @@
         <v>21.67</v>
       </c>
       <c r="F35" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1167,7 +1164,7 @@
         <v>10.19</v>
       </c>
       <c r="F37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1204,7 +1201,7 @@
         <v>8.6</v>
       </c>
       <c r="F39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1241,7 +1238,7 @@
         <v>15.54</v>
       </c>
       <c r="F41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1286,7 +1283,7 @@
         <v>6.8</v>
       </c>
       <c r="C44" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D44">
         <v>0</v>
@@ -1354,7 +1351,7 @@
         <v>14.5</v>
       </c>
       <c r="C48" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -1380,7 +1377,7 @@
         <v>64.06</v>
       </c>
       <c r="F49" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -1425,7 +1422,7 @@
         <v>5.8</v>
       </c>
       <c r="C52" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -1485,7 +1482,7 @@
         <v>64.099999999999994</v>
       </c>
       <c r="F55" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>